<commit_message>
Release gate first, in priority order: high-risk leaks, precision, invented text, cost
</commit_message>
<xml_diff>
--- a/results/jev_haiku_test_run.xlsx
+++ b/results/jev_haiku_test_run.xlsx
@@ -33656,17 +33656,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2. Invented text (Haiku items not in the chat)</t>
+          <t>2. Precision (extracted items that are real PII, all categories)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>over 90%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>95.8% (69/72)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -33678,17 +33678,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>3. Cost per 1,000 chats (Jev + Haiku)</t>
+          <t>3. Invented text (Haiku items not in the chat)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>under $0.50</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>$0.261</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -33700,17 +33700,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>4. Precision (extracted items that are real PII, all categories)</t>
+          <t>4. Cost per 1,000 chats (Jev + Haiku)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>over 90%</t>
+          <t>under $0.50</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>95.8% (69/72)</t>
+          <t>$0.261</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">

</xml_diff>